<commit_message>
fix: entry multiple data
</commit_message>
<xml_diff>
--- a/imports/templates/mining_productions_import_template.xlsx
+++ b/imports/templates/mining_productions_import_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10315"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10503"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/meinardus/Documents/template-import/alpha-mines/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/meinardus/Project/python/mines-smart/imports/templates/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B671D3BC-7486-0949-87CC-DD7561033488}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C766FB6C-0DE2-2446-A2A5-7AE3E7957152}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="880" windowWidth="36000" windowHeight="20820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20" yWindow="880" windowWidth="36000" windowHeight="20820" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="productions" sheetId="1" r:id="rId1"/>
@@ -177,9 +177,6 @@
     <t>Quarry</t>
   </si>
   <si>
-    <t>dome</t>
-  </si>
-  <si>
     <t>block_id</t>
   </si>
   <si>
@@ -208,6 +205,9 @@
   </si>
   <si>
     <t>DT-263-NPM</t>
+  </si>
+  <si>
+    <t>pile_id</t>
   </si>
 </sst>
 </file>
@@ -759,7 +759,7 @@
         <v>30</v>
       </c>
       <c r="E1" s="16" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="F1" s="12" t="s">
         <v>38</v>
@@ -768,19 +768,19 @@
         <v>39</v>
       </c>
       <c r="H1" s="17" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="I1" s="12" t="s">
         <v>40</v>
       </c>
       <c r="J1" s="12" t="s">
+        <v>48</v>
+      </c>
+      <c r="K1" s="18" t="s">
         <v>49</v>
       </c>
-      <c r="K1" s="18" t="s">
-        <v>50</v>
-      </c>
       <c r="L1" s="14" t="s">
-        <v>47</v>
+        <v>57</v>
       </c>
       <c r="M1" s="14" t="s">
         <v>29</v>
@@ -792,13 +792,13 @@
         <v>41</v>
       </c>
       <c r="P1" s="14" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="Q1" s="14" t="s">
+        <v>50</v>
+      </c>
+      <c r="R1" s="14" t="s">
         <v>51</v>
-      </c>
-      <c r="R1" s="14" t="s">
-        <v>52</v>
       </c>
       <c r="S1" s="14" t="s">
         <v>33</v>
@@ -827,7 +827,7 @@
         <v>0.875</v>
       </c>
       <c r="F2" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G2" s="23">
         <v>5</v>
@@ -836,13 +836,13 @@
         <v>45</v>
       </c>
       <c r="I2" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J2" s="24" t="s">
         <v>36</v>
       </c>
       <c r="K2" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L2" s="25"/>
       <c r="M2" s="24" t="s">
@@ -872,7 +872,7 @@
         <v>0.875</v>
       </c>
       <c r="F3" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G3" s="23">
         <v>5</v>
@@ -881,13 +881,13 @@
         <v>45</v>
       </c>
       <c r="I3" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J3" s="24" t="s">
         <v>36</v>
       </c>
       <c r="K3" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L3" s="25"/>
       <c r="M3" s="24" t="s">
@@ -917,7 +917,7 @@
         <v>0.875</v>
       </c>
       <c r="F4" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G4" s="23">
         <v>5</v>
@@ -926,13 +926,13 @@
         <v>45</v>
       </c>
       <c r="I4" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J4" s="24" t="s">
         <v>36</v>
       </c>
       <c r="K4" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L4" s="25"/>
       <c r="M4" s="24" t="s">
@@ -962,7 +962,7 @@
         <v>0.875</v>
       </c>
       <c r="F5" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G5" s="23">
         <v>5</v>
@@ -971,13 +971,13 @@
         <v>45</v>
       </c>
       <c r="I5" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J5" s="24" t="s">
         <v>36</v>
       </c>
       <c r="K5" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L5" s="25"/>
       <c r="M5" s="24" t="s">
@@ -1007,7 +1007,7 @@
         <v>0.875</v>
       </c>
       <c r="F6" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G6" s="23">
         <v>5</v>
@@ -1016,13 +1016,13 @@
         <v>45</v>
       </c>
       <c r="I6" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J6" s="24" t="s">
         <v>36</v>
       </c>
       <c r="K6" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L6" s="25"/>
       <c r="M6" s="24" t="s">
@@ -1052,7 +1052,7 @@
         <v>0.875</v>
       </c>
       <c r="F7" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G7" s="23">
         <v>5</v>
@@ -1061,13 +1061,13 @@
         <v>45</v>
       </c>
       <c r="I7" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J7" s="24" t="s">
         <v>36</v>
       </c>
       <c r="K7" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L7" s="25"/>
       <c r="M7" s="24" t="s">
@@ -1097,7 +1097,7 @@
         <v>0.875</v>
       </c>
       <c r="F8" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G8" s="23">
         <v>5</v>
@@ -1106,13 +1106,13 @@
         <v>45</v>
       </c>
       <c r="I8" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J8" s="24" t="s">
         <v>36</v>
       </c>
       <c r="K8" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L8" s="25"/>
       <c r="M8" s="24" t="s">
@@ -1142,7 +1142,7 @@
         <v>0.875</v>
       </c>
       <c r="F9" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G9" s="23">
         <v>5</v>
@@ -1151,13 +1151,13 @@
         <v>45</v>
       </c>
       <c r="I9" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J9" s="24" t="s">
         <v>36</v>
       </c>
       <c r="K9" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L9" s="25"/>
       <c r="M9" s="24" t="s">
@@ -1187,7 +1187,7 @@
         <v>0.875</v>
       </c>
       <c r="F10" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G10" s="23">
         <v>5</v>
@@ -1196,13 +1196,13 @@
         <v>45</v>
       </c>
       <c r="I10" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J10" s="24" t="s">
         <v>36</v>
       </c>
       <c r="K10" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L10" s="25"/>
       <c r="M10" s="24" t="s">
@@ -1232,7 +1232,7 @@
         <v>0.875</v>
       </c>
       <c r="F11" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G11" s="23">
         <v>5</v>
@@ -1241,13 +1241,13 @@
         <v>45</v>
       </c>
       <c r="I11" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J11" s="24" t="s">
         <v>36</v>
       </c>
       <c r="K11" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L11" s="25"/>
       <c r="M11" s="24" t="s">
@@ -1277,7 +1277,7 @@
         <v>0.875</v>
       </c>
       <c r="F12" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G12" s="23">
         <v>5</v>
@@ -1286,13 +1286,13 @@
         <v>45</v>
       </c>
       <c r="I12" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J12" s="24" t="s">
         <v>36</v>
       </c>
       <c r="K12" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L12" s="25"/>
       <c r="M12" s="24" t="s">
@@ -1322,7 +1322,7 @@
         <v>0.875</v>
       </c>
       <c r="F13" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G13" s="23">
         <v>5</v>
@@ -1331,13 +1331,13 @@
         <v>45</v>
       </c>
       <c r="I13" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J13" s="24" t="s">
         <v>36</v>
       </c>
       <c r="K13" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L13" s="25"/>
       <c r="M13" s="24" t="s">
@@ -1367,7 +1367,7 @@
         <v>0.875</v>
       </c>
       <c r="F14" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G14" s="23">
         <v>5</v>
@@ -1376,13 +1376,13 @@
         <v>45</v>
       </c>
       <c r="I14" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J14" s="24" t="s">
         <v>36</v>
       </c>
       <c r="K14" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L14" s="25"/>
       <c r="M14" s="24" t="s">
@@ -1412,7 +1412,7 @@
         <v>0.875</v>
       </c>
       <c r="F15" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G15" s="23">
         <v>5</v>
@@ -1421,13 +1421,13 @@
         <v>45</v>
       </c>
       <c r="I15" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J15" s="24" t="s">
         <v>36</v>
       </c>
       <c r="K15" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L15" s="25"/>
       <c r="M15" s="24" t="s">
@@ -1457,7 +1457,7 @@
         <v>0.875</v>
       </c>
       <c r="F16" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G16" s="23">
         <v>5</v>
@@ -1466,13 +1466,13 @@
         <v>45</v>
       </c>
       <c r="I16" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J16" s="24" t="s">
         <v>36</v>
       </c>
       <c r="K16" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L16" s="25"/>
       <c r="M16" s="24" t="s">
@@ -1502,7 +1502,7 @@
         <v>0.875</v>
       </c>
       <c r="F17" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G17" s="23">
         <v>5</v>
@@ -1511,13 +1511,13 @@
         <v>45</v>
       </c>
       <c r="I17" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J17" s="24" t="s">
         <v>36</v>
       </c>
       <c r="K17" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L17" s="25"/>
       <c r="M17" s="24" t="s">
@@ -1547,7 +1547,7 @@
         <v>0.875</v>
       </c>
       <c r="F18" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G18" s="23">
         <v>5</v>
@@ -1556,13 +1556,13 @@
         <v>45</v>
       </c>
       <c r="I18" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J18" s="24" t="s">
         <v>36</v>
       </c>
       <c r="K18" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L18" s="25"/>
       <c r="M18" s="24" t="s">
@@ -1592,7 +1592,7 @@
         <v>0.875</v>
       </c>
       <c r="F19" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G19" s="23">
         <v>5</v>
@@ -1601,13 +1601,13 @@
         <v>45</v>
       </c>
       <c r="I19" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J19" s="24" t="s">
         <v>36</v>
       </c>
       <c r="K19" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L19" s="25"/>
       <c r="M19" s="24" t="s">
@@ -1637,7 +1637,7 @@
         <v>0.875</v>
       </c>
       <c r="F20" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G20" s="23">
         <v>5</v>
@@ -1646,13 +1646,13 @@
         <v>45</v>
       </c>
       <c r="I20" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J20" s="24" t="s">
         <v>36</v>
       </c>
       <c r="K20" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L20" s="25"/>
       <c r="M20" s="24" t="s">
@@ -1682,7 +1682,7 @@
         <v>0.875</v>
       </c>
       <c r="F21" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G21" s="23">
         <v>5</v>
@@ -1691,13 +1691,13 @@
         <v>45</v>
       </c>
       <c r="I21" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J21" s="24" t="s">
         <v>36</v>
       </c>
       <c r="K21" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L21" s="25"/>
       <c r="M21" s="24" t="s">
@@ -1727,7 +1727,7 @@
         <v>0.875</v>
       </c>
       <c r="F22" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G22" s="23">
         <v>5</v>
@@ -1736,13 +1736,13 @@
         <v>45</v>
       </c>
       <c r="I22" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J22" s="24" t="s">
         <v>36</v>
       </c>
       <c r="K22" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L22" s="25"/>
       <c r="M22" s="24" t="s">
@@ -1772,7 +1772,7 @@
         <v>0.875</v>
       </c>
       <c r="F23" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G23" s="23">
         <v>5</v>
@@ -1781,13 +1781,13 @@
         <v>45</v>
       </c>
       <c r="I23" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J23" s="24" t="s">
         <v>36</v>
       </c>
       <c r="K23" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L23" s="25"/>
       <c r="M23" s="24" t="s">
@@ -1817,7 +1817,7 @@
         <v>0.875</v>
       </c>
       <c r="F24" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G24" s="23">
         <v>5</v>
@@ -1826,13 +1826,13 @@
         <v>45</v>
       </c>
       <c r="I24" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J24" s="24" t="s">
         <v>36</v>
       </c>
       <c r="K24" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L24" s="25"/>
       <c r="M24" s="24" t="s">
@@ -1862,7 +1862,7 @@
         <v>0.875</v>
       </c>
       <c r="F25" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G25" s="23">
         <v>5</v>
@@ -1871,13 +1871,13 @@
         <v>45</v>
       </c>
       <c r="I25" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J25" s="24" t="s">
         <v>36</v>
       </c>
       <c r="K25" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L25" s="25"/>
       <c r="M25" s="24" t="s">
@@ -1907,7 +1907,7 @@
         <v>0.875</v>
       </c>
       <c r="F26" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G26" s="23">
         <v>5</v>
@@ -1916,13 +1916,13 @@
         <v>45</v>
       </c>
       <c r="I26" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J26" s="24" t="s">
         <v>36</v>
       </c>
       <c r="K26" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L26" s="25"/>
       <c r="M26" s="24" t="s">
@@ -1952,7 +1952,7 @@
         <v>0.875</v>
       </c>
       <c r="F27" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G27" s="23">
         <v>5</v>
@@ -1961,13 +1961,13 @@
         <v>45</v>
       </c>
       <c r="I27" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J27" s="24" t="s">
         <v>36</v>
       </c>
       <c r="K27" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L27" s="25"/>
       <c r="M27" s="24" t="s">
@@ -1997,7 +1997,7 @@
         <v>0.875</v>
       </c>
       <c r="F28" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G28" s="23">
         <v>5</v>
@@ -2006,13 +2006,13 @@
         <v>45</v>
       </c>
       <c r="I28" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J28" s="24" t="s">
         <v>36</v>
       </c>
       <c r="K28" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L28" s="25"/>
       <c r="M28" s="24" t="s">
@@ -2042,7 +2042,7 @@
         <v>0.875</v>
       </c>
       <c r="F29" s="22" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="G29" s="23">
         <v>5</v>
@@ -2051,13 +2051,13 @@
         <v>45</v>
       </c>
       <c r="I29" s="24" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="J29" s="24" t="s">
         <v>36</v>
       </c>
       <c r="K29" s="25" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="L29" s="25"/>
       <c r="M29" s="24" t="s">

</xml_diff>